<commit_message>
feat: improve enquiry form and lead management
</commit_message>
<xml_diff>
--- a/enquiries.xlsx
+++ b/enquiries.xlsx
@@ -3,6 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+  </bookViews>
   <sheets>
     <sheet sheetId="1" name="Enquiries" state="visible" r:id="rId4"/>
   </sheets>
@@ -11,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="51">
   <si>
     <t>Enquiry ID</t>
   </si>
@@ -28,22 +31,118 @@
     <t>Email</t>
   </si>
   <si>
+    <t>Lead Type</t>
+  </si>
+  <si>
+    <t>Enquiry Type</t>
+  </si>
+  <si>
+    <t>GSTIN</t>
+  </si>
+  <si>
+    <t>Event Type</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Event Date</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
     <t>Address</t>
   </si>
   <si>
-    <t>Lead Type</t>
-  </si>
-  <si>
-    <t>Enquiry Type</t>
+    <t>Message</t>
   </si>
   <si>
     <t>ENQ0001</t>
   </si>
   <si>
-    <t>22-08-2026 14:08:12</t>
-  </si>
-  <si>
-    <t>Karthikeya Thammishetti</t>
+    <t>01-09-2026 08:17:48</t>
+  </si>
+  <si>
+    <t>Browser User Test</t>
+  </si>
+  <si>
+    <t>9123456789</t>
+  </si>
+  <si>
+    <t>browseruser@example.com</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>Corporate Gifting</t>
+  </si>
+  <si>
+    <t>36TEST1234F1Z0</t>
+  </si>
+  <si>
+    <t>Corporate</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>2026-11-05</t>
+  </si>
+  <si>
+    <t>500/kit</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Testing submission to live server on port 3000</t>
+  </si>
+  <si>
+    <t>ENQ0002</t>
+  </si>
+  <si>
+    <t>01-09-2026 08:18:05</t>
+  </si>
+  <si>
+    <t>Radhika Sharma</t>
+  </si>
+  <si>
+    <t>9876501234</t>
+  </si>
+  <si>
+    <t>radhika@example.com</t>
+  </si>
+  <si>
+    <t>Bulk Orders</t>
+  </si>
+  <si>
+    <t>36RADH1234F1Z1</t>
+  </si>
+  <si>
+    <t>Wedding</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>2026-11-25</t>
+  </si>
+  <si>
+    <t>250/piece</t>
+  </si>
+  <si>
+    <t>Dry fruit hampers with velvet box packing</t>
+  </si>
+  <si>
+    <t>ENQ0003</t>
+  </si>
+  <si>
+    <t>01-09-2026 08:18:38</t>
+  </si>
+  <si>
+    <t>Karthikeya</t>
   </si>
   <si>
     <t>+917386699734</t>
@@ -52,25 +151,22 @@
     <t>thammishettikarthikeya@gmail.com</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>Personal Gifting, Bulk Orders</t>
-  </si>
-  <si>
-    <t>ENQ0002</t>
-  </si>
-  <si>
-    <t>22-08-2026 14:13:51</t>
-  </si>
-  <si>
     <t>Wholesaler</t>
   </si>
   <si>
-    <t>Personal Gifting, Bulk Orders, Corporate Gifting</t>
+    <t>Hydrabad</t>
+  </si>
+  <si>
+    <t>ENQ0004</t>
+  </si>
+  <si>
+    <t>01-09-2026 08:22:18</t>
+  </si>
+  <si>
+    <t>+917386699732</t>
+  </si>
+  <si>
+    <t>Personal Gifting</t>
   </si>
 </sst>
 </file>
@@ -87,6 +183,8 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -451,8 +549,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -464,7 +562,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -489,57 +587,199 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" t="s">
+        <v>46</v>
+      </c>
+      <c r="N4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L5" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" t="s">
+        <v>46</v>
+      </c>
+      <c r="N5" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>